<commit_message>
auto update 2026-10-15 11:08 UTC
</commit_message>
<xml_diff>
--- a/exports/project120_polls.xlsx
+++ b/exports/project120_polls.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'כל התוצאות (ארוך)'!$A$1:$M$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'מכונים'!$A$1:$C$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ערוצי פרסום'!$A$1:$D$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'רשומות הוועדה (גולמי)'!$A$1:$J$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'רשומות הוועדה (גולמי)'!$A$1:$J$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J109"/>
+  <dimension ref="A1:J110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5720,8 +5720,36 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>4209</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="n"/>
+      <c r="C110" s="2" t="n"/>
+      <c r="D110" s="2" t="n"/>
+      <c r="E110" s="2" t="n"/>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="n"/>
+      <c r="H110" s="2" t="n"/>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>Survey4209.pdf</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gov.il/BlobFolder/dynamiccollectorresultitem/knesset_election108/he/Survey4209.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J109"/>
+  <autoFilter ref="A1:J110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
auto update 2026-10-15 16:01 UTC
</commit_message>
<xml_diff>
--- a/exports/project120_polls.xlsx
+++ b/exports/project120_polls.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'כל התוצאות (ארוך)'!$A$1:$M$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'מכונים'!$A$1:$C$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ערוצי פרסום'!$A$1:$D$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'רשומות הוועדה (גולמי)'!$A$1:$J$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'רשומות הוועדה (גולמי)'!$A$1:$J$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J110"/>
+  <dimension ref="A1:J111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5748,8 +5748,36 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>4210</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="n"/>
+      <c r="C111" s="2" t="n"/>
+      <c r="D111" s="2" t="n"/>
+      <c r="E111" s="2" t="n"/>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="n"/>
+      <c r="H111" s="2" t="n"/>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>Survey_4210.pdf</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gov.il/BlobFolder/dynamiccollectorresultitem/knesset_election109/he/Survey_4210.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J110"/>
+  <autoFilter ref="A1:J111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
auto update 2026-10-16 10:04 UTC
</commit_message>
<xml_diff>
--- a/exports/project120_polls.xlsx
+++ b/exports/project120_polls.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'כל התוצאות (ארוך)'!$A$1:$M$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'מכונים'!$A$1:$C$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ערוצי פרסום'!$A$1:$D$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'רשומות הוועדה (גולמי)'!$A$1:$J$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'רשומות הוועדה (גולמי)'!$A$1:$J$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J111"/>
+  <dimension ref="A1:J113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5776,8 +5776,64 @@
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>4211</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="n"/>
+      <c r="C112" s="2" t="n"/>
+      <c r="D112" s="2" t="n"/>
+      <c r="E112" s="2" t="n"/>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="n"/>
+      <c r="H112" s="2" t="n"/>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>Survey_4211.pdf</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gov.il/BlobFolder/dynamiccollectorresultitem/knesset_election110/he/Survey_4211.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>4212</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="n"/>
+      <c r="C113" s="2" t="n"/>
+      <c r="D113" s="2" t="n"/>
+      <c r="E113" s="2" t="n"/>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="n"/>
+      <c r="H113" s="2" t="n"/>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>Survey_4212.pdf</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gov.il/BlobFolder/dynamiccollectorresultitem/knesset_election111/he/Survey_4212.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J111"/>
+  <autoFilter ref="A1:J113"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>